<commit_message>
Update Grupo + link Github.xlsx file
Replaced the existing Grupo + link Github.xlsx file with a new version. The update may include changes to group information or GitHub links.
</commit_message>
<xml_diff>
--- a/Grupo + link Github.xlsx
+++ b/Grupo + link Github.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felip\Escritorio\Capstone\Capstone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felip\Escritorio\Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D7698FC-8651-4CA4-878C-191E07BAEEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48FF70B4-6F81-4193-BFC9-0CA316065E59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CB75DAD0-5A7E-4FD9-8750-010779140108}"/>
   </bookViews>
@@ -170,11 +170,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -187,8 +188,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{CE0638DF-DF68-4A46-A27B-98C40F9E5C81}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -522,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A69A014-F2D7-4AB1-B9EF-0139B87CC8EA}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.28515625" customWidth="1"/>
@@ -576,7 +579,7 @@
       <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="6" t="s">
         <v>10</v>
       </c>
     </row>
@@ -599,7 +602,7 @@
       <c r="F3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="6" t="s">
         <v>10</v>
       </c>
     </row>
@@ -622,11 +625,19 @@
       <c r="F4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="6" t="s">
         <v>10</v>
       </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G6" s="3"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{D5B9294E-8A98-4848-9FAF-8668BD7C7019}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{E034A9B7-7E4C-4DA9-8F39-787F528759F6}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{A5B4584C-431B-4EF7-B3D2-6DD0912B58B7}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>